<commit_message>
aggiornamento 2026 09 28 15:21
</commit_message>
<xml_diff>
--- a/AntonioCristiano/Template mappatura anno 2.xlsx
+++ b/AntonioCristiano/Template mappatura anno 2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RickyMandich\PROJECT\appuntiITS\AntonioCristiano\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A87C1DFB-D45E-4481-AC26-12BFC53FDF09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{277D8AB1-28C1-4D73-8F54-89408FBF7BFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="36">
   <si>
     <t>Nome azienda</t>
   </si>
@@ -43,9 +43,6 @@
     <t>posizioni aperte</t>
   </si>
   <si>
-    <t>Vai Software</t>
-  </si>
-  <si>
     <t>vaisoftware.it</t>
   </si>
   <si>
@@ -55,9 +52,6 @@
     <t>info@vaisoftware.it</t>
   </si>
   <si>
-    <t>Piazza Aldo Moro 10</t>
-  </si>
-  <si>
     <t>il sito non dispone di questa pagina</t>
   </si>
   <si>
@@ -73,17 +67,74 @@
     <t>sipe@sipe.it</t>
   </si>
   <si>
-    <t>Via Colombo</t>
-  </si>
-  <si>
     <t>Java senior developer, Programmatore iSeries, Analista Programmatore iSeries</t>
+  </si>
+  <si>
+    <t>rubynetti</t>
+  </si>
+  <si>
+    <t>rubynetti.it</t>
+  </si>
+  <si>
+    <t>info@rubynetti.it</t>
+  </si>
+  <si>
+    <t>42 bit</t>
+  </si>
+  <si>
+    <t>42b.it</t>
+  </si>
+  <si>
+    <t>349 3250613</t>
+  </si>
+  <si>
+    <t>info@42b.it</t>
+  </si>
+  <si>
+    <t>via della Libertà, 12 - 30175</t>
+  </si>
+  <si>
+    <t>IT support specialist</t>
+  </si>
+  <si>
+    <t>Calle dei Furlani, 30122 Castello</t>
+  </si>
+  <si>
+    <t>Via Colombo 4, 30037 scorzè</t>
+  </si>
+  <si>
+    <t>Vai S.R.L</t>
+  </si>
+  <si>
+    <t>Piazza Aldo Moro 10 - 35129 padova</t>
+  </si>
+  <si>
+    <t>didanet</t>
+  </si>
+  <si>
+    <t>didanet.org</t>
+  </si>
+  <si>
+    <t>049 7800645</t>
+  </si>
+  <si>
+    <t>info@didanet.org</t>
+  </si>
+  <si>
+    <t>Via dell’Elettricità 5/D, 30175 Marghera</t>
+  </si>
+  <si>
+    <t>Full stack developer</t>
+  </si>
+  <si>
+    <t>priorità</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -99,6 +150,20 @@
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -121,15 +186,19 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -346,79 +415,191 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultColWidth="19.88671875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="33.21875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="66.88671875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2">
+        <v>4679760282</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="1">
+        <v>4026430274</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4">
+        <v>3248500278</v>
+      </c>
+      <c r="D4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5">
+        <v>4225940271</v>
+      </c>
+      <c r="D5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6">
+        <v>4565180280</v>
+      </c>
+      <c r="D6" t="s">
         <v>7</v>
       </c>
-      <c r="B2">
-        <v>4565180280</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="E6" t="s">
         <v>8</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F6" t="s">
         <v>9</v>
       </c>
-      <c r="E2" t="s">
+      <c r="G6" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="H6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B3">
-        <v>3248500278</v>
-      </c>
-      <c r="C3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" t="s">
-        <v>17</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>18</v>
-      </c>
+    </row>
+    <row r="7" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="2"/>
+      <c r="F7" s="3"/>
+      <c r="H7" s="2"/>
+    </row>
+    <row r="8" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="2"/>
+      <c r="F8" s="3"/>
+      <c r="H8" s="2"/>
+    </row>
+    <row r="9" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="2"/>
+      <c r="F9" s="3"/>
+      <c r="H9" s="2"/>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H6">
+    <sortCondition ref="A2:A6"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>